<commit_message>
[main] Migrate gem to skill
</commit_message>
<xml_diff>
--- a/ia/Fulvito.xlsx
+++ b/ia/Fulvito.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="44">
   <si>
     <t>Fecha</t>
   </si>
@@ -109,10 +109,10 @@
     <t>Santi</t>
   </si>
   <si>
-    <t>Tomas</t>
+    <t>Tizi</t>
   </si>
   <si>
-    <t>Will</t>
+    <t>Tomas</t>
   </si>
   <si>
     <t>A</t>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t>Xavi</t>
+  </si>
+  <si>
+    <t>Will</t>
   </si>
   <si>
     <t>E</t>
@@ -412,7 +415,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F171" displayName="Fulvito" name="Fulvito" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F191" displayName="Fulvito" name="Fulvito" id="1">
   <tableColumns count="6">
     <tableColumn name="Fecha" id="1"/>
     <tableColumn name="Partido #" id="2"/>
@@ -426,7 +429,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="H1:M25" displayName="Estadisticas" name="Estadisticas" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="H1:M26" displayName="Estadisticas" name="Estadisticas" id="2">
   <tableColumns count="6">
     <tableColumn name="Jugador" id="1"/>
     <tableColumn name="Partidos" id="2"/>
@@ -822,32 +825,32 @@
         <v>15.0</v>
       </c>
       <c r="H2" s="11" t="str">
-        <f t="array" ref="H2:H26">SORT(UNIQUE(C2:C1120))</f>
+        <f t="array" ref="H2:H27">SORT(UNIQUE(C2:C1140))</f>
         <v>Alf</v>
       </c>
       <c r="I2" s="12">
-        <f t="shared" ref="I2:I25" si="1">COUNTIF($C$2:$C$1120, H2)</f>
-        <v>16</v>
+        <f t="shared" ref="I2:I26" si="1">COUNTIF($C$2:$C$1140, H2)</f>
+        <v>18</v>
       </c>
       <c r="J2" s="13">
-        <f t="shared" ref="J2:J25" si="2">COUNTIFS($C$2:$C$1120, H2, $E$2:$E$1120, "V")
+        <f t="shared" ref="J2:J26" si="2">COUNTIFS($C$2:$C$1140, H2, $E$2:$E$1140, "V")
 </f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K2" s="13">
-        <f t="shared" ref="K2:K25" si="3">COUNTIFS($C$2:$C$1120, H2, $E$2:$E$1120, "E")</f>
+        <f t="shared" ref="K2:K26" si="3">COUNTIFS($C$2:$C$1140, H2, $E$2:$E$1140, "E")</f>
         <v>3</v>
       </c>
       <c r="L2" s="13">
-        <f t="shared" ref="L2:L25" si="4">COUNTIFS($C$2:$C$1120, H2, $E$2:$E$1120, "D")</f>
-        <v>7</v>
+        <f t="shared" ref="L2:L26" si="4">COUNTIFS($C$2:$C$1140, H2, $E$2:$E$1140, "D")</f>
+        <v>8</v>
       </c>
       <c r="M2" s="14">
-        <f t="shared" ref="M2:M25" si="5">IFERROR(J2/I2, 0)</f>
-        <v>0.375</v>
+        <f t="shared" ref="M2:M26" si="5">IFERROR(J2/I2, 0)</f>
+        <v>0.3888888889</v>
       </c>
       <c r="O2" s="15" t="str">
-        <f t="array" ref="O2:O26">SORT(UNIQUE(C2:C1120))</f>
+        <f t="array" ref="O2:O27">SORT(UNIQUE(C2:C1140))</f>
         <v>Alf</v>
       </c>
       <c r="P2" s="16" t="s">
@@ -860,8 +863,8 @@
       <c r="S2" s="18" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("LET(
   jugs, H2:H24,
-  p_equipos, FILTER(B2:B1128 &amp; ""_"" &amp; UPPER(TRIM(D2:D1128)), C2:C1128&lt;&gt;""""),
-  nombres, FILTER(C2:C1128, C2:C1128&lt;&gt;""""),
+  p_equipos, FILTER(B2:B1148 &amp; ""_"" &amp; UPPER(TRIM(D2:D1148)), C2:C1148&lt;&gt;""""),
+  nombres, FILTER(C2:C1148, C2:C1148&lt;&gt;""""),
   unicos, UNIQUE(p_equipos),
   U, ARRAYFORMULA(--(unicos = TRANSPOSE(p_equipos))),
   P, ARRAYFORMULA(--(nombre"&amp;"s = TRANSPOSE(jugs))),
@@ -880,8 +883,8 @@
         <v>0</v>
       </c>
       <c r="V2" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
       </c>
       <c r="W2" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -896,8 +899,8 @@
         <v>0</v>
       </c>
       <c r="Z2" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="AA2" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -924,16 +927,16 @@
         <v>0</v>
       </c>
       <c r="AG2" s="18">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
+        <v>6</v>
+      </c>
+      <c r="AH2" s="18">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
+      </c>
+      <c r="AI2" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
         <v>5</v>
-      </c>
-      <c r="AH2" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
-      </c>
-      <c r="AI2" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
       </c>
       <c r="AJ2" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
@@ -956,8 +959,8 @@
         <v>1</v>
       </c>
       <c r="AO2" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
@@ -1272,7 +1275,7 @@
       </c>
       <c r="I5" s="12">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J5" s="13">
         <f t="shared" si="2"/>
@@ -1284,11 +1287,11 @@
       </c>
       <c r="L5" s="13">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M5" s="14">
         <f t="shared" si="5"/>
-        <v>0.3333333333</v>
+        <v>0.2727272727</v>
       </c>
       <c r="O5" s="20" t="s">
         <v>14</v>
@@ -1300,8 +1303,8 @@
         <v>14</v>
       </c>
       <c r="S5" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
       </c>
       <c r="T5" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -1316,8 +1319,8 @@
         <v>-</v>
       </c>
       <c r="W5" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="X5" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -1328,8 +1331,8 @@
         <v>1</v>
       </c>
       <c r="Z5" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="AA5" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
@@ -1340,8 +1343,8 @@
         <v>0</v>
       </c>
       <c r="AC5" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="AD5" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -1360,20 +1363,20 @@
         <v>6</v>
       </c>
       <c r="AH5" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
       </c>
       <c r="AI5" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="AJ5" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
         <v>4</v>
       </c>
       <c r="AK5" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="AL5" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -1416,7 +1419,7 @@
       </c>
       <c r="I6" s="12">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" s="13">
         <f t="shared" si="2"/>
@@ -1428,7 +1431,7 @@
       </c>
       <c r="L6" s="13">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" s="14">
         <f t="shared" si="5"/>
@@ -1456,8 +1459,8 @@
         <v>0</v>
       </c>
       <c r="V6" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="W6" s="18" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"-")</f>
@@ -1472,8 +1475,8 @@
         <v>0</v>
       </c>
       <c r="Z6" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="AA6" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -1484,8 +1487,8 @@
         <v>0</v>
       </c>
       <c r="AC6" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="AD6" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -1516,8 +1519,8 @@
         <v>0</v>
       </c>
       <c r="AK6" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="AL6" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -1848,7 +1851,7 @@
       </c>
       <c r="I9" s="12">
         <f t="shared" si="1"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J9" s="13">
         <f t="shared" si="2"/>
@@ -1860,11 +1863,11 @@
       </c>
       <c r="L9" s="13">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M9" s="14">
         <f t="shared" si="5"/>
-        <v>0.3571428571</v>
+        <v>0.3125</v>
       </c>
       <c r="O9" s="20" t="s">
         <v>18</v>
@@ -1876,8 +1879,8 @@
         <v>18</v>
       </c>
       <c r="S9" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="T9" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -1888,12 +1891,12 @@
         <v>1</v>
       </c>
       <c r="V9" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="W9" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="X9" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -1916,8 +1919,8 @@
         <v>2</v>
       </c>
       <c r="AC9" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
       </c>
       <c r="AD9" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -1936,20 +1939,20 @@
         <v>6</v>
       </c>
       <c r="AH9" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
-        <v>8</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
+        <v>9</v>
       </c>
       <c r="AI9" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="AJ9" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
         <v>6</v>
       </c>
       <c r="AK9" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
+        <v>6</v>
       </c>
       <c r="AL9" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -1964,8 +1967,8 @@
         <v>0</v>
       </c>
       <c r="AO9" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
@@ -2280,11 +2283,11 @@
       </c>
       <c r="I12" s="12">
         <f t="shared" si="1"/>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J12" s="13">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K12" s="13">
         <f t="shared" si="3"/>
@@ -2292,7 +2295,7 @@
       </c>
       <c r="L12" s="13">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M12" s="14">
         <f t="shared" si="5"/>
@@ -2302,7 +2305,7 @@
         <v>21</v>
       </c>
       <c r="P12" s="16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="R12" s="17" t="s">
         <v>21</v>
@@ -2320,12 +2323,12 @@
         <v>0</v>
       </c>
       <c r="V12" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="W12" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="X12" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
@@ -2336,8 +2339,8 @@
         <v>1</v>
       </c>
       <c r="Z12" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
       </c>
       <c r="AA12" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
@@ -2364,8 +2367,8 @@
         <v>2</v>
       </c>
       <c r="AG12" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
-        <v>6</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
       </c>
       <c r="AH12" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
@@ -2376,28 +2379,28 @@
         <v>2</v>
       </c>
       <c r="AJ12" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
-      </c>
-      <c r="AK12" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
         <v>8</v>
       </c>
+      <c r="AK12" s="18">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.0)</f>
+        <v>10</v>
+      </c>
       <c r="AL12" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
         <v>1</v>
       </c>
       <c r="AM12" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="AN12" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="AO12" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
@@ -2856,11 +2859,11 @@
       </c>
       <c r="I16" s="12">
         <f t="shared" si="1"/>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J16" s="13">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K16" s="22">
         <f t="shared" si="3"/>
@@ -2872,7 +2875,7 @@
       </c>
       <c r="M16" s="23">
         <f t="shared" si="5"/>
-        <v>0.3125</v>
+        <v>0.3888888889</v>
       </c>
       <c r="O16" s="20" t="s">
         <v>25</v>
@@ -2884,8 +2887,8 @@
         <v>25</v>
       </c>
       <c r="S16" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
+        <v>6</v>
       </c>
       <c r="T16" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -2924,8 +2927,8 @@
         <v>1</v>
       </c>
       <c r="AC16" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
-        <v>6</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
       </c>
       <c r="AD16" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
@@ -2944,36 +2947,36 @@
         <v>-</v>
       </c>
       <c r="AH16" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
-      </c>
-      <c r="AI16" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
-      </c>
-      <c r="AJ16" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
-        <v>9</v>
-      </c>
-      <c r="AK16" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
         <v>6</v>
       </c>
-      <c r="AL16" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
-      </c>
-      <c r="AM16" s="18">
+      <c r="AI16" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
         <v>2</v>
       </c>
+      <c r="AJ16" s="18">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.0)</f>
+        <v>10</v>
+      </c>
+      <c r="AK16" s="18">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
+      </c>
+      <c r="AL16" s="18">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
+      </c>
+      <c r="AM16" s="18">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
+      </c>
       <c r="AN16" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="AO16" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
@@ -3000,11 +3003,11 @@
       </c>
       <c r="I17" s="12">
         <f t="shared" si="1"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J17" s="22">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K17" s="22">
         <f t="shared" si="3"/>
@@ -3012,11 +3015,11 @@
       </c>
       <c r="L17" s="22">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M17" s="23">
         <f t="shared" si="5"/>
-        <v>0.5714285714</v>
+        <v>0.5625</v>
       </c>
       <c r="O17" s="20" t="s">
         <v>26</v>
@@ -3028,8 +3031,8 @@
         <v>26</v>
       </c>
       <c r="S17" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
       </c>
       <c r="T17" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -3040,8 +3043,8 @@
         <v>0</v>
       </c>
       <c r="V17" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
+        <v>4</v>
       </c>
       <c r="W17" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -3056,8 +3059,8 @@
         <v>0</v>
       </c>
       <c r="Z17" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
-        <v>8</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
+        <v>9</v>
       </c>
       <c r="AA17" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -3084,16 +3087,16 @@
         <v>2</v>
       </c>
       <c r="AG17" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
+        <v>6</v>
       </c>
       <c r="AH17" s="18" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"-")</f>
         <v>-</v>
       </c>
       <c r="AI17" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
       </c>
       <c r="AJ17" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
@@ -3144,11 +3147,11 @@
       </c>
       <c r="I18" s="12">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J18" s="22">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K18" s="22">
         <f t="shared" si="3"/>
@@ -3156,11 +3159,11 @@
       </c>
       <c r="L18" s="22">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M18" s="23">
         <f t="shared" si="5"/>
-        <v>0.25</v>
+        <v>0.3333333333</v>
       </c>
       <c r="O18" s="20" t="s">
         <v>27</v>
@@ -3172,8 +3175,8 @@
         <v>27</v>
       </c>
       <c r="S18" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
-        <v>3</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="T18" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -3184,8 +3187,8 @@
         <v>0</v>
       </c>
       <c r="V18" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="W18" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -3200,8 +3203,8 @@
         <v>0</v>
       </c>
       <c r="Z18" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="AA18" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -3228,12 +3231,12 @@
         <v>0</v>
       </c>
       <c r="AG18" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="AH18" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
       </c>
       <c r="AI18" s="18" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"-")</f>
@@ -3256,8 +3259,8 @@
         <v>1</v>
       </c>
       <c r="AN18" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="AO18" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -3288,11 +3291,11 @@
       </c>
       <c r="I19" s="12">
         <f t="shared" si="1"/>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J19" s="22">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K19" s="22">
         <f t="shared" si="3"/>
@@ -3304,7 +3307,7 @@
       </c>
       <c r="M19" s="23">
         <f t="shared" si="5"/>
-        <v>0.4705882353</v>
+        <v>0.5</v>
       </c>
       <c r="O19" s="20" t="s">
         <v>28</v>
@@ -3356,8 +3359,8 @@
         <v>2</v>
       </c>
       <c r="AC19" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
+        <v>8</v>
       </c>
       <c r="AD19" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
@@ -3372,8 +3375,8 @@
         <v>4</v>
       </c>
       <c r="AG19" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
-        <v>9</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.0)</f>
+        <v>10</v>
       </c>
       <c r="AH19" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
@@ -3388,16 +3391,16 @@
         <v>-</v>
       </c>
       <c r="AK19" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
-        <v>9</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.0)</f>
+        <v>10</v>
       </c>
       <c r="AL19" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
         <v>0</v>
       </c>
       <c r="AM19" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="AN19" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -3432,11 +3435,11 @@
       </c>
       <c r="I20" s="12">
         <f t="shared" si="1"/>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J20" s="22">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K20" s="22">
         <f t="shared" si="3"/>
@@ -3444,11 +3447,11 @@
       </c>
       <c r="L20" s="22">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M20" s="23">
         <f t="shared" si="5"/>
-        <v>0.4705882353</v>
+        <v>0.4736842105</v>
       </c>
       <c r="O20" s="20" t="s">
         <v>29</v>
@@ -3472,12 +3475,12 @@
         <v>0</v>
       </c>
       <c r="V20" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="W20" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
+        <v>2</v>
       </c>
       <c r="X20" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
@@ -3488,8 +3491,8 @@
         <v>0</v>
       </c>
       <c r="Z20" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
-        <v>5</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
+        <v>6</v>
       </c>
       <c r="AA20" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -3500,8 +3503,8 @@
         <v>2</v>
       </c>
       <c r="AC20" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
-        <v>8</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.0)</f>
+        <v>10</v>
       </c>
       <c r="AD20" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -3516,8 +3519,8 @@
         <v>2</v>
       </c>
       <c r="AG20" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
-        <v>6</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
+        <v>7</v>
       </c>
       <c r="AH20" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
@@ -3528,8 +3531,8 @@
         <v>2</v>
       </c>
       <c r="AJ20" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
-        <v>9</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.0)</f>
+        <v>10</v>
       </c>
       <c r="AK20" s="18" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"-")</f>
@@ -3540,16 +3543,16 @@
         <v>0</v>
       </c>
       <c r="AM20" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
+        <v>8</v>
       </c>
       <c r="AN20" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="AO20" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
@@ -3720,11 +3723,11 @@
       </c>
       <c r="I22" s="12">
         <f t="shared" si="1"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J22" s="22">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K22" s="22">
         <f t="shared" si="3"/>
@@ -3736,7 +3739,7 @@
       </c>
       <c r="M22" s="23">
         <f t="shared" si="5"/>
-        <v>0.4615384615</v>
+        <v>0.5</v>
       </c>
       <c r="O22" s="20" t="s">
         <v>31</v>
@@ -3788,8 +3791,8 @@
         <v>1</v>
       </c>
       <c r="AC22" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="AD22" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -3804,8 +3807,8 @@
         <v>0</v>
       </c>
       <c r="AG22" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
-        <v>2</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
+        <v>3</v>
       </c>
       <c r="AH22" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),6.0)</f>
@@ -3816,12 +3819,12 @@
         <v>1</v>
       </c>
       <c r="AJ22" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4.0)</f>
-        <v>4</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),5.0)</f>
+        <v>5</v>
       </c>
       <c r="AK22" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),7.0)</f>
-        <v>7</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
+        <v>8</v>
       </c>
       <c r="AL22" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2.0)</f>
@@ -3868,11 +3871,11 @@
       </c>
       <c r="J23" s="22">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" s="22">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" s="22">
         <f t="shared" si="4"/>
@@ -3880,7 +3883,7 @@
       </c>
       <c r="M23" s="23">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23" s="20" t="s">
         <v>32</v>
@@ -3932,8 +3935,8 @@
         <v>0</v>
       </c>
       <c r="AC23" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="AD23" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -3948,24 +3951,24 @@
         <v>0</v>
       </c>
       <c r="AG23" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="AH23" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
         <v>1</v>
       </c>
       <c r="AI23" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="AJ23" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
         <v>0</v>
       </c>
       <c r="AK23" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="AL23" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -4012,11 +4015,11 @@
       </c>
       <c r="J24" s="22">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" s="22">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="22">
         <f t="shared" si="4"/>
@@ -4024,20 +4027,20 @@
       </c>
       <c r="M24" s="23">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" s="20" t="s">
         <v>33</v>
       </c>
       <c r="P24" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R24" s="17" t="s">
         <v>33</v>
       </c>
       <c r="S24" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="T24" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -4064,8 +4067,8 @@
         <v>0</v>
       </c>
       <c r="Z24" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="AA24" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -4076,8 +4079,8 @@
         <v>0</v>
       </c>
       <c r="AC24" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="AD24" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -4092,8 +4095,8 @@
         <v>0</v>
       </c>
       <c r="AG24" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="AH24" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
@@ -4108,8 +4111,8 @@
         <v>0</v>
       </c>
       <c r="AK24" s="18">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
-        <v>0</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),1.0)</f>
+        <v>1</v>
       </c>
       <c r="AL24" s="18">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
@@ -4148,11 +4151,11 @@
         <v>8.0</v>
       </c>
       <c r="H25" s="21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I25" s="12">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J25" s="22">
         <f t="shared" si="2"/>
@@ -4164,14 +4167,14 @@
       </c>
       <c r="L25" s="22">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M25" s="23">
         <f t="shared" si="5"/>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="O25" s="20" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P25" s="16" t="s">
         <v>37</v>
@@ -4196,8 +4199,35 @@
       <c r="F26" s="7">
         <v>12.0</v>
       </c>
-      <c r="H26" s="24"/>
-      <c r="O26" s="24"/>
+      <c r="H26" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="I26" s="12">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="J26" s="22">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="K26" s="22">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="L26" s="22">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="M26" s="23">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="O26" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="P26" s="16" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="27" ht="22.5" customHeight="1">
       <c r="A27" s="6">
@@ -4218,6 +4248,8 @@
       <c r="F27" s="7">
         <v>12.0</v>
       </c>
+      <c r="H27" s="24"/>
+      <c r="O27" s="24"/>
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="6">
@@ -5313,7 +5345,7 @@
         <v>34</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F82" s="7">
         <v>14.0</v>
@@ -5333,7 +5365,7 @@
         <v>34</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F83" s="7">
         <v>14.0</v>
@@ -5353,7 +5385,7 @@
         <v>34</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F84" s="7">
         <v>14.0</v>
@@ -5373,7 +5405,7 @@
         <v>34</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F85" s="7">
         <v>14.0</v>
@@ -5393,7 +5425,7 @@
         <v>34</v>
       </c>
       <c r="E86" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F86" s="7">
         <v>14.0</v>
@@ -5413,7 +5445,7 @@
         <v>37</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F87" s="7">
         <v>14.0</v>
@@ -5433,7 +5465,7 @@
         <v>37</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F88" s="7">
         <v>14.0</v>
@@ -5453,7 +5485,7 @@
         <v>37</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F89" s="7">
         <v>14.0</v>
@@ -5473,7 +5505,7 @@
         <v>37</v>
       </c>
       <c r="E90" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F90" s="7">
         <v>14.0</v>
@@ -5493,7 +5525,7 @@
         <v>37</v>
       </c>
       <c r="E91" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F91" s="7">
         <v>14.0</v>
@@ -6487,7 +6519,7 @@
         <v>14.0</v>
       </c>
       <c r="C141" s="8" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D141" s="9" t="s">
         <v>37</v>
@@ -6713,7 +6745,7 @@
         <v>34</v>
       </c>
       <c r="E152" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F152" s="7">
         <v>7.0</v>
@@ -6733,7 +6765,7 @@
         <v>34</v>
       </c>
       <c r="E153" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F153" s="7">
         <v>7.0</v>
@@ -6753,7 +6785,7 @@
         <v>34</v>
       </c>
       <c r="E154" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F154" s="7">
         <v>7.0</v>
@@ -6770,10 +6802,10 @@
         <v>18</v>
       </c>
       <c r="D155" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E155" s="8" t="s">
         <v>42</v>
-      </c>
-      <c r="E155" s="8" t="s">
-        <v>41</v>
       </c>
       <c r="F155" s="7">
         <v>7.0</v>
@@ -6793,7 +6825,7 @@
         <v>34</v>
       </c>
       <c r="E156" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F156" s="7">
         <v>7.0</v>
@@ -6813,7 +6845,7 @@
         <v>37</v>
       </c>
       <c r="E157" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F157" s="7">
         <v>7.0</v>
@@ -6833,7 +6865,7 @@
         <v>37</v>
       </c>
       <c r="E158" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F158" s="7">
         <v>7.0</v>
@@ -6853,7 +6885,7 @@
         <v>37</v>
       </c>
       <c r="E159" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F159" s="7">
         <v>7.0</v>
@@ -6873,7 +6905,7 @@
         <v>37</v>
       </c>
       <c r="E160" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F160" s="7">
         <v>7.0</v>
@@ -6887,13 +6919,13 @@
         <v>16.0</v>
       </c>
       <c r="C161" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D161" s="9" t="s">
         <v>37</v>
       </c>
       <c r="E161" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F161" s="7">
         <v>7.0</v>
@@ -6913,7 +6945,7 @@
         <v>34</v>
       </c>
       <c r="E162" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F162" s="7">
         <v>13.0</v>
@@ -6933,7 +6965,7 @@
         <v>34</v>
       </c>
       <c r="E163" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F163" s="7">
         <v>13.0</v>
@@ -6953,7 +6985,7 @@
         <v>34</v>
       </c>
       <c r="E164" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F164" s="7">
         <v>13.0</v>
@@ -6973,7 +7005,7 @@
         <v>34</v>
       </c>
       <c r="E165" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F165" s="7">
         <v>13.0</v>
@@ -6993,7 +7025,7 @@
         <v>34</v>
       </c>
       <c r="E166" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F166" s="7">
         <v>13.0</v>
@@ -7013,7 +7045,7 @@
         <v>37</v>
       </c>
       <c r="E167" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F167" s="7">
         <v>13.0</v>
@@ -7033,7 +7065,7 @@
         <v>37</v>
       </c>
       <c r="E168" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F168" s="7">
         <v>13.0</v>
@@ -7053,7 +7085,7 @@
         <v>37</v>
       </c>
       <c r="E169" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F169" s="7">
         <v>13.0</v>
@@ -7073,7 +7105,7 @@
         <v>37</v>
       </c>
       <c r="E170" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F170" s="7">
         <v>13.0</v>
@@ -7093,33 +7125,433 @@
         <v>37</v>
       </c>
       <c r="E171" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F171" s="7">
         <v>13.0</v>
       </c>
     </row>
+    <row r="172" ht="22.5" customHeight="1">
+      <c r="A172" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B172" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C172" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D172" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E172" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F172" s="7">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="173" ht="22.5" customHeight="1">
+      <c r="A173" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B173" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C173" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D173" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E173" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F173" s="7">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="174" ht="22.5" customHeight="1">
+      <c r="A174" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B174" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C174" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D174" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E174" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F174" s="7">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="175" ht="22.5" customHeight="1">
+      <c r="A175" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B175" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C175" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D175" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E175" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F175" s="7">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="176" ht="22.5" customHeight="1">
+      <c r="A176" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B176" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C176" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D176" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E176" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F176" s="7">
+        <v>10.0</v>
+      </c>
+    </row>
+    <row r="177" ht="22.5" customHeight="1">
+      <c r="A177" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B177" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C177" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D177" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E177" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F177" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="178" ht="22.5" customHeight="1">
+      <c r="A178" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B178" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C178" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D178" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E178" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F178" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="179" ht="22.5" customHeight="1">
+      <c r="A179" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B179" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C179" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D179" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E179" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F179" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="180" ht="22.5" customHeight="1">
+      <c r="A180" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B180" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C180" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D180" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E180" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F180" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="181" ht="22.5" customHeight="1">
+      <c r="A181" s="25">
+        <v>46267.0</v>
+      </c>
+      <c r="B181" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="C181" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D181" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E181" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F181" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="182" ht="22.5" customHeight="1">
+      <c r="A182" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B182" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C182" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D182" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E182" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F182" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="183" ht="22.5" customHeight="1">
+      <c r="A183" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B183" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C183" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D183" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E183" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F183" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="184" ht="22.5" customHeight="1">
+      <c r="A184" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B184" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C184" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D184" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E184" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F184" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="185" ht="22.5" customHeight="1">
+      <c r="A185" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B185" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C185" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D185" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E185" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F185" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="186" ht="22.5" customHeight="1">
+      <c r="A186" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B186" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C186" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D186" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E186" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F186" s="7">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="187" ht="22.5" customHeight="1">
+      <c r="A187" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B187" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C187" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D187" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E187" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F187" s="7">
+        <v>14.0</v>
+      </c>
+    </row>
+    <row r="188" ht="22.5" customHeight="1">
+      <c r="A188" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B188" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C188" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D188" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E188" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F188" s="7">
+        <v>14.0</v>
+      </c>
+    </row>
+    <row r="189" ht="22.5" customHeight="1">
+      <c r="A189" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B189" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C189" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D189" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E189" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F189" s="7">
+        <v>14.0</v>
+      </c>
+    </row>
+    <row r="190" ht="22.5" customHeight="1">
+      <c r="A190" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B190" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C190" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D190" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E190" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F190" s="7">
+        <v>14.0</v>
+      </c>
+    </row>
+    <row r="191" ht="22.5" customHeight="1">
+      <c r="A191" s="25">
+        <v>46295.0</v>
+      </c>
+      <c r="B191" s="7">
+        <v>19.0</v>
+      </c>
+      <c r="C191" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D191" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E191" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F191" s="7">
+        <v>14.0</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A171">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A191">
       <formula1>OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="B2:B171 F2:F171">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="B2:B191 F2:F191">
       <formula1>AND(ISNUMBER(B2),(NOT(OR(NOT(ISERROR(DATEVALUE(B2))), AND(ISNUMBER(B2), LEFT(CELL("format", B2))="D")))))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="P2:P25">
+    <dataValidation type="list" allowBlank="1" sqref="P2:P26">
       <formula1>"A,B,C,D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="E2:E171">
+    <dataValidation type="list" allowBlank="1" sqref="E2:E191">
       <formula1>"V,V,V,V,V,D,D,D,D,D,V,V,E"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:M25">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="I2:M26">
       <formula1>AND(ISNUMBER(I2),(NOT(OR(NOT(ISERROR(DATEVALUE(I2))), AND(ISNUMBER(I2), LEFT(CELL("format", I2))="D")))))</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="H2:H25"/>
-    <dataValidation type="list" allowBlank="1" sqref="C2:C171">
-      <formula1>"NicoRz,Ema,Mauri,Odri,Fede,Leo,Ivan,Marce,Mauro,Alf,Santi,Xavi,Facu,Mateo,Franquito,Manuelo,Juan,NicoL,Ruso,Will,Colo,Duki,Tomas,Fabri"</formula1>
+    <dataValidation type="list" allowBlank="1" sqref="C2:C191">
+      <formula1>"NicoRz,Ema,Mauri,Odri,Fede,Leo,Ivan,Marce,Mauro,Alf,Santi,Xavi,Facu,Mateo,Franquito,Manuelo,Juan,NicoL,Ruso,Will,Colo,Duki,Tomas,Fabri,Tizi"</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showDropDown="1" sqref="H2:H26"/>
   </dataValidations>
   <drawing r:id="rId1"/>
   <tableParts count="3">

</xml_diff>